<commit_message>
Align the demo schedule and attendance files and document the rules
</commit_message>
<xml_diff>
--- a/docs/demo/cedvel.xlsx
+++ b/docs/demo/cedvel.xlsx
@@ -449,7 +449,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1">
-        <v>46321.0</v>
+        <v>46300.0</v>
       </c>
       <c r="B2" s="2">
         <v>0.79166666666667</v>
@@ -467,7 +467,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1">
-        <v>46323.0</v>
+        <v>46302.0</v>
       </c>
       <c r="B3" s="2">
         <v>0.79166666666667</v>
@@ -485,7 +485,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1">
-        <v>46325.0</v>
+        <v>46304.0</v>
       </c>
       <c r="B4" s="2">
         <v>0.79166666666667</v>
@@ -503,7 +503,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1">
-        <v>46328.0</v>
+        <v>46307.0</v>
       </c>
       <c r="B5" s="2">
         <v>0.79166666666667</v>
@@ -521,7 +521,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1">
-        <v>46330.0</v>
+        <v>46309.0</v>
       </c>
       <c r="B6" s="2">
         <v>0.79166666666667</v>
@@ -539,7 +539,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1">
-        <v>46332.0</v>
+        <v>46311.0</v>
       </c>
       <c r="B7" s="2">
         <v>0.79166666666667</v>
@@ -557,7 +557,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1">
-        <v>46335.0</v>
+        <v>46314.0</v>
       </c>
       <c r="B8" s="2">
         <v>0.79166666666667</v>
@@ -575,7 +575,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1">
-        <v>46337.0</v>
+        <v>46316.0</v>
       </c>
       <c r="B9" s="2">
         <v>0.79166666666667</v>
@@ -593,7 +593,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1">
-        <v>46339.0</v>
+        <v>46318.0</v>
       </c>
       <c r="B10" s="2">
         <v>0.79166666666667</v>
@@ -611,7 +611,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1">
-        <v>46342.0</v>
+        <v>46321.0</v>
       </c>
       <c r="B11" s="2">
         <v>0.79166666666667</v>
@@ -629,7 +629,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1">
-        <v>46344.0</v>
+        <v>46323.0</v>
       </c>
       <c r="B12" s="2">
         <v>0.79166666666667</v>
@@ -647,7 +647,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1">
-        <v>46346.0</v>
+        <v>46325.0</v>
       </c>
       <c r="B13" s="2">
         <v>0.79166666666667</v>

</xml_diff>